<commit_message>
Import TEM-4 pack 17 (9.26) words and images.
Bring 201 new exam entries and JPEGs online so the production static CDN and vocab seed stay in sync.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/content/senses_table_tem8_merged.xlsx
+++ b/data/content/senses_table_tem8_merged.xlsx
@@ -581,7 +581,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ortografía</t>
+          <t>convención</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -601,22 +601,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>拼写</t>
+          <t>协议；约定</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Cuidar la ortografía incluye tildes y la diferencia entre b/v o g/j según la regla.</t>
+          <t>Los dos países firmaron una convención para proteger el medio ambiente y los recursos naturales.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>注意拼写包括重音符号，以及按规则区分 b/v、g/j 等。</t>
+          <t>两国签署了一项保护环境和自然资源的协议。</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>images/ortografia_1.jpg</t>
+          <t>images/convencion_1.jpg</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -628,7 +628,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>presupuesto</t>
+          <t>escala</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -648,22 +648,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>预算</t>
+          <t>梯子；阶梯</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Haz un presupuesto mensual: comida, transporte, material de estudio y un pequeño ahorro.</t>
+          <t>Los pintores usaron una escala para alcanzar la parte alta de la pared del aula.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>做一份月预算：吃饭、交通、学习用品和一点储蓄。</t>
+          <t>油漆工用梯子够到教室墙壁的高处。</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>images/presupuesto_1.jpg</t>
+          <t>images/escala_1.jpg</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -675,7 +675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>traducción</t>
+          <t>estabilidad</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -695,22 +695,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>翻译</t>
+          <t>稳定；稳固；持久性</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>La traducción no es solo cambiar palabras: hay que respetar el sentido y el tono del texto original.</t>
+          <t>La estabilidad económica es fundamental para que los estudiantes puedan terminar sus carreras.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>翻译不只是换词，还要尊重原文的意义与语气。</t>
+          <t>经济稳定对学生完成学业至关重要。</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>images/traduccion_1.jpg</t>
+          <t>images/estabilidad_1.jpg</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -722,7 +722,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>acusación</t>
+          <t>evidencia</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -737,39 +737,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>指控；控告</t>
+          <t>明显；证据</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>La acusación carece de pruebas suficientes.</t>
+          <t>No hay evidencia de que el examen fuera demasiado difícil para los estudiantes.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>该指控缺乏足够证据。</t>
+          <t>没有证据表明考试对学生来说太难了。</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>images/acusacion_1.jpg</t>
+          <t>images/evidencia_1.jpg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>afirmación</t>
+          <t>exposición</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -784,39 +784,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>断言；肯定说法</t>
+          <t>阐述；陈述；展览</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Su afirmación no se sostiene con los datos.</t>
+          <t>La exposición clara de las hipótesis de trabajo es fundamental para lograr una buena nota en la defensa.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>他的断言得不到数据支撑。</t>
+          <t>清晰地阐述工作假说是为了在答辩中取得好成绩的关键基础。</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>images/afirmacion_1.jpg</t>
+          <t>images/exposicion_1.jpg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>alusión</t>
+          <t>interpretación</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -831,39 +831,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>暗指；典故式提及</t>
+          <t>口译；阐释；理解</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>El texto hace una alusión a Cervantes.</t>
+          <t>La interpretación de los textos antiguos requiere un profundo conocimiento de la cultura de la época.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>文本暗指塞万提斯。</t>
+          <t>对古籍的阐释需要对那个时代的文化有深刻的了解。</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>images/alusion_1.jpg</t>
+          <t>images/interpretacion_1.jpg</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>analogía</t>
+          <t>ortografía</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -878,39 +878,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>类比</t>
+          <t>拼写</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Usa una analogía para explicar el concepto.</t>
+          <t>Cuidar la ortografía incluye tildes y la diferencia entre b/v o g/j según la regla.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>他用类比解释该概念。</t>
+          <t>注意拼写包括重音符号，以及按规则区分 b/v、g/j 等。</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>images/analogia_1.jpg</t>
+          <t>images/ortografia_1.jpg</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>anexo</t>
+          <t>presupuesto</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -925,39 +925,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>附录</t>
+          <t>预算</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Los datos completos figuran en el anexo.</t>
+          <t>Haz un presupuesto mensual: comida, transporte, material de estudio y un pequeño ahorro.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>完整数据见附录。</t>
+          <t>做一份月预算：吃饭、交通、学习用品和一点储蓄。</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>images/anexo_1.jpg</t>
+          <t>images/presupuesto_1.jpg</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>antonimia</t>
+          <t>traducción</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -972,39 +972,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>反义关系</t>
+          <t>翻译</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Alto/bajo es un ejemplo clásico de antonimia gradable.</t>
+          <t>La traducción no es solo cambiar palabras: hay que respetar el sentido y el tono del texto original.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>高/低是典型的可分级反义。</t>
+          <t>翻译不只是换词，还要尊重原文的意义与语气。</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>images/antonimia_1.jpg</t>
+          <t>images/traduccion_1.jpg</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>análisis</t>
+          <t>acusación</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1024,34 +1024,34 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>分析</t>
+          <t>指控；控告</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>El análisis del discurso revela cómo los conectores organizan la argumentación en un editorial.</t>
+          <t>La acusación carece de pruebas suficientes.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>话语分析揭示连接词如何在社论中组织论证结构。</t>
+          <t>该指控缺乏足够证据。</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>images/analisis_1.jpg</t>
+          <t>images/acusacion_1.jpg</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>专八|专四</t>
+          <t>专八</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>aproximación</t>
+          <t>afirmación</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1071,22 +1071,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>方法；进路；接近</t>
+          <t>断言；肯定说法</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Proponemos una aproximación interdisciplinaria.</t>
+          <t>Su afirmación no se sostiene con los datos.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>我们提出跨学科进路。</t>
+          <t>他的断言得不到数据支撑。</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>images/aproximacion_1.jpg</t>
+          <t>images/afirmacion_1.jpg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>argumentación</t>
+          <t>alusión</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1118,22 +1118,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>论证；论述</t>
+          <t>暗指；典故式提及</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>La argumentación del ensayo debe presentar pruebas y contraargumentos.</t>
+          <t>El texto hace una alusión a Cervantes.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>论文的论证应提出证据与反驳。</t>
+          <t>文本暗指塞万提斯。</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>images/argumentacion_1.jpg</t>
+          <t>images/alusion_1.jpg</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1145,7 +1145,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>arqueología</t>
+          <t>analogía</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1165,22 +1165,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>考古学</t>
+          <t>类比</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>La arqueología aporta datos materiales sobre el pasado.</t>
+          <t>Usa una analogía para explicar el concepto.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>考古学为过去提供物质证据。</t>
+          <t>他用类比解释该概念。</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>images/arqueologia_1.jpg</t>
+          <t>images/analogia_1.jpg</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1192,7 +1192,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>artefacto</t>
+          <t>anexo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1212,22 +1212,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>人工制品；产物</t>
+          <t>附录</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>El texto es un artefacto cultural de su época.</t>
+          <t>Los datos completos figuran en el anexo.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>文本是其时代的文化产物。</t>
+          <t>完整数据见附录。</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>images/artefacto_1.jpg</t>
+          <t>images/anexo_1.jpg</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bilingüismo</t>
+          <t>antonimia</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1259,22 +1259,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>双语能力；双语现象</t>
+          <t>反义关系</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>El bilingüismo no implica dominio perfecto de ambas lenguas en todos los registros.</t>
+          <t>Alto/bajo es un ejemplo clásico de antonimia gradable.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>双语并不意味着两种语言在一切语体上都完美精通。</t>
+          <t>高/低是典型的可分级反义。</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>images/bilinguismo_1.jpg</t>
+          <t>images/antonimia_1.jpg</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1286,7 +1286,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>categoría</t>
+          <t>análisis</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1306,34 +1306,34 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>范畴；类别</t>
+          <t>分析</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Hay que definir cada categoría con precisión.</t>
+          <t>El análisis del discurso revela cómo los conectores organizan la argumentación en un editorial.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>必须精确界定每一范畴。</t>
+          <t>话语分析揭示连接词如何在社论中组织论证结构。</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>images/categoria_1.jpg</t>
+          <t>images/analisis_1.jpg</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>causalidad</t>
+          <t>aproximación</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1353,22 +1353,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>因果关系</t>
+          <t>方法；进路；接近</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Correlación no implica necesariamente causalidad.</t>
+          <t>Proponemos una aproximación interdisciplinaria.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>相关并不必然意味着因果。</t>
+          <t>我们提出跨学科进路。</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>images/causalidad_1.jpg</t>
+          <t>images/aproximacion_1.jpg</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1380,7 +1380,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cláusula</t>
+          <t>argumentación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1400,22 +1400,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>从句；条款</t>
+          <t>论证；论述</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Analiza la cláusula subordinada del periodo.</t>
+          <t>La argumentación del ensayo debe presentar pruebas y contraargumentos.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>分析该句中的从属从句。</t>
+          <t>论文的论证应提出证据与反驳。</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>images/clausula_1.jpg</t>
+          <t>images/argumentacion_1.jpg</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>codificación</t>
+          <t>arqueología</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1447,22 +1447,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>编码</t>
+          <t>考古学</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>La codificación de los datos sigue un protocolo.</t>
+          <t>La arqueología aporta datos materiales sobre el pasado.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>数据编码遵循协议。</t>
+          <t>考古学为过去提供物质证据。</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>images/codificacion_1.jpg</t>
+          <t>images/arqueologia_1.jpg</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1474,7 +1474,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cognición</t>
+          <t>artefacto</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1494,22 +1494,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>认知</t>
+          <t>人工制品；产物</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>La cognición humana procesa el lenguaje en red.</t>
+          <t>El texto es un artefacto cultural de su época.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>人类认知以网络方式处理语言。</t>
+          <t>文本是其时代的文化产物。</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>images/cognicion_1.jpg</t>
+          <t>images/artefacto_1.jpg</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1521,7 +1521,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>coherencia</t>
+          <t>bilingüismo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1541,22 +1541,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>连贯；条理</t>
+          <t>双语能力；双语现象</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>La coherencia textual depende de que cada párrafo avance la idea central sin contradicciones.</t>
+          <t>El bilingüismo no implica dominio perfecto de ambas lenguas en todos los registros.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>篇章连贯取决于每一段推进中心思想且不自相矛盾。</t>
+          <t>双语并不意味着两种语言在一切语体上都完美精通。</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>images/coherencia_1.jpg</t>
+          <t>images/bilinguismo_1.jpg</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1568,7 +1568,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cohesión</t>
+          <t>categoría</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1588,22 +1588,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>衔接（语言学术语）</t>
+          <t>范畴；类别</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Los pronombres y los conectores aportan cohesión al unir oraciones dentro del mismo párrafo.</t>
+          <t>Hay que definir cada categoría con precisión.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>代词与连接词通过把句间关系连起来，带来篇章衔接。</t>
+          <t>必须精确界定每一范畴。</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>images/cohesion_1.jpg</t>
+          <t>images/categoria_1.jpg</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1615,7 +1615,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>colonización</t>
+          <t>causalidad</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1635,22 +1635,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>殖民</t>
+          <t>因果关系</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>La colonización dejó huellas lingüísticas profundas.</t>
+          <t>Correlación no implica necesariamente causalidad.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>殖民留下深刻的语言痕迹。</t>
+          <t>相关并不必然意味着因果。</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>images/colonizacion_1.jpg</t>
+          <t>images/causalidad_1.jpg</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1662,7 +1662,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>competencia</t>
+          <t>cláusula</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1682,22 +1682,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>能力；（语言）能力</t>
+          <t>从句；条款</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>La competencia comunicativa incluye saber qué decir, cómo decirlo y cuándo callar.</t>
+          <t>Analiza la cláusula subordinada del periodo.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>交际能力包括知道说什么、怎么说，以及何时保持沉默。</t>
+          <t>分析该句中的从属从句。</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>images/competencia_1.jpg</t>
+          <t>images/clausula_1.jpg</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1709,12 +1709,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>competencia</t>
+          <t>codificación</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1729,22 +1729,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>竞争；竞赛</t>
+          <t>编码</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>La competencia entre empresas tecnológicas acelera la innovación, pero también genera presión laboral.</t>
+          <t>La codificación de los datos sigue un protocolo.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>科技企业间的竞争加速创新，但也带来职场压力。</t>
+          <t>数据编码遵循协议。</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>images/competencia_2.jpg</t>
+          <t>images/codificacion_1.jpg</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1756,7 +1756,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>complejidad</t>
+          <t>cognición</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1776,22 +1776,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>复杂性</t>
+          <t>认知</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>La complejidad del fenómeno exige varios enfoques.</t>
+          <t>La cognición humana procesa el lenguaje en red.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>现象的复杂性要求多种方法。</t>
+          <t>人类认知以网络方式处理语言。</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>images/complejidad_1.jpg</t>
+          <t>images/cognicion_1.jpg</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1803,7 +1803,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>compromiso</t>
+          <t>coherencia</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1823,22 +1823,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>承诺；介入</t>
+          <t>连贯；条理</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>El texto muestra un compromiso ético.</t>
+          <t>La coherencia textual depende de que cada párrafo avance la idea central sin contradicciones.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>文本显示出伦理介入。</t>
+          <t>篇章连贯取决于每一段推进中心思想且不自相矛盾。</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>images/compromiso_1.jpg</t>
+          <t>images/coherencia_1.jpg</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1850,7 +1850,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>conciliación</t>
+          <t>cohesión</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1870,22 +1870,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>调解；和解</t>
+          <t>衔接（语言学术语）</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Buscan la conciliación de intereses opuestos.</t>
+          <t>Los pronombres y los conectores aportan cohesión al unir oraciones dentro del mismo párrafo.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>他们寻求对立利益的和解。</t>
+          <t>代词与连接词通过把句间关系连起来，带来篇章衔接。</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>images/conciliacion_1.jpg</t>
+          <t>images/cohesion_1.jpg</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1897,7 +1897,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>conclusión</t>
+          <t>colonización</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1917,22 +1917,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>结论</t>
+          <t>殖民</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>En la conclusión no introduzcas datos nuevos; resume y señala límites o futuras líneas de trabajo.</t>
+          <t>La colonización dejó huellas lingüísticas profundas.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>结论部分不要引入新数据；应总结并指出局限或未来研究方向。</t>
+          <t>殖民留下深刻的语言痕迹。</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>images/conclusion_1.jpg</t>
+          <t>images/colonizacion_1.jpg</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1944,7 +1944,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>configuración</t>
+          <t>competencia</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1964,22 +1964,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>构型；配置</t>
+          <t>能力；（语言）能力</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Analizamos la configuración del relato.</t>
+          <t>La competencia comunicativa incluye saber qué decir, cómo decirlo y cuándo callar.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>我们分析叙事构型。</t>
+          <t>交际能力包括知道说什么、怎么说，以及何时保持沉默。</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>images/configuracion_1.jpg</t>
+          <t>images/competencia_1.jpg</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1991,12 +1991,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>consenso</t>
+          <t>competencia</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2011,22 +2011,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>共识</t>
+          <t>竞争；竞赛</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>No hay consenso sobre la definición.</t>
+          <t>La competencia entre empresas tecnológicas acelera la innovación, pero también genera presión laboral.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>关于定义尚无共识。</t>
+          <t>科技企业间的竞争加速创新，但也带来职场压力。</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>images/consenso_1.jpg</t>
+          <t>images/competencia_2.jpg</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2038,7 +2038,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>consistencia</t>
+          <t>complejidad</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2058,22 +2058,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>一致性；连贯严谨</t>
+          <t>复杂性</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>La consistencia argumentativa es esencial.</t>
+          <t>La complejidad del fenómeno exige varios enfoques.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>论证一致性至关重要。</t>
+          <t>现象的复杂性要求多种方法。</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>images/consistencia_1.jpg</t>
+          <t>images/complejidad_1.jpg</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2085,7 +2085,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>contaminación</t>
+          <t>compromiso</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2105,22 +2105,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>污染；（也指）干扰</t>
+          <t>承诺；介入</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Hay contaminación entre variedades en contacto.</t>
+          <t>El texto muestra un compromiso ético.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>接触中的变体之间存在干扰。</t>
+          <t>文本显示出伦理介入。</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>images/contaminacion_1.jpg</t>
+          <t>images/compromiso_1.jpg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2132,7 +2132,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>contextualizar</t>
+          <t>conciliación</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>v</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2152,22 +2152,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>置于语境；语境化</t>
+          <t>调解；和解</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Hay que contextualizar la cita antes de analizarla.</t>
+          <t>Buscan la conciliación de intereses opuestos.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>分析引文前须先置于语境。</t>
+          <t>他们寻求对立利益的和解。</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>images/contextualizar_1.jpg</t>
+          <t>images/conciliacion_1.jpg</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2179,7 +2179,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>contradicción</t>
+          <t>conclusión</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2199,22 +2199,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>矛盾</t>
+          <t>结论</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>El texto cae en contradicción entre el primer y el último párrafo.</t>
+          <t>En la conclusión no introduzcas datos nuevos; resume y señala límites o futuras líneas de trabajo.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>文本在首段与末段之间自相矛盾。</t>
+          <t>结论部分不要引入新数据；应总结并指出局限或未来研究方向。</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>images/contradiccion_1.jpg</t>
+          <t>images/conclusion_1.jpg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>contraposición</t>
+          <t>configuración</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2246,22 +2246,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>对照；对立设置</t>
+          <t>构型；配置</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>La contraposición de personajes estructura la novela.</t>
+          <t>Analizamos la configuración del relato.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>人物对照构成小说结构。</t>
+          <t>我们分析叙事构型。</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>images/contraposicion_1.jpg</t>
+          <t>images/configuracion_1.jpg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2273,7 +2273,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>convención</t>
+          <t>consenso</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2293,22 +2293,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>惯例；公约</t>
+          <t>共识</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Rompe la convención narrativa del final cerrado.</t>
+          <t>No hay consenso sobre la definición.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>它打破封闭结局的叙事惯例。</t>
+          <t>关于定义尚无共识。</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>images/convencion_1.jpg</t>
+          <t>images/consenso_1.jpg</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2320,7 +2320,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>correlación</t>
+          <t>consistencia</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2340,22 +2340,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>相关；相关性</t>
+          <t>一致性；连贯严谨</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Hay correlación entre horas de estudio y rendimiento.</t>
+          <t>La consistencia argumentativa es esencial.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>学习时长与成绩之间存在相关。</t>
+          <t>论证一致性至关重要。</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>images/correlacion_1.jpg</t>
+          <t>images/consistencia_1.jpg</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>corroborar</t>
+          <t>contaminación</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>v</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2387,22 +2387,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>证实；确证</t>
+          <t>污染；（也指）干扰</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Los datos corroboran la hipótesis.</t>
+          <t>Hay contaminación entre variedades en contacto.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>数据证实了该假设。</t>
+          <t>接触中的变体之间存在干扰。</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>images/corroborar_1.jpg</t>
+          <t>images/contaminacion_1.jpg</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2414,7 +2414,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>credibilidad</t>
+          <t>contextualizar</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>v</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2434,22 +2434,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>可信度</t>
+          <t>置于语境；语境化</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>La fuente pierde credibilidad sin referencias.</t>
+          <t>Hay que contextualizar la cita antes de analizarla.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>缺少出处会降低来源可信度。</t>
+          <t>分析引文前须先置于语境。</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>images/credibilidad_1.jpg</t>
+          <t>images/contextualizar_1.jpg</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>criterio</t>
+          <t>contradicción</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2481,34 +2481,34 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>标准；准则</t>
+          <t>矛盾</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Hay que definir criterios claros de evaluación.</t>
+          <t>El texto cae en contradicción entre el primer y el último párrafo.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>必须明确评价标准。</t>
+          <t>文本在首段与末段之间自相矛盾。</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>images/criterio_1.jpg</t>
+          <t>images/contradiccion_1.jpg</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>专八|专四</t>
+          <t>专八</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>crítica</t>
+          <t>contraposición</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2528,22 +2528,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>评论；批评</t>
+          <t>对照；对立设置</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>La crítica literaria no solo juzga si un libro «gusta», sino cómo construye sentido y estilo.</t>
+          <t>La contraposición de personajes estructura la novela.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>文学批评不只判断书是否「好看」，还分析它如何构建意义与风格。</t>
+          <t>人物对照构成小说结构。</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>images/critica_1.jpg</t>
+          <t>images/contraposicion_1.jpg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2555,7 +2555,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cuestionario</t>
+          <t>correlación</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2575,22 +2575,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>问卷</t>
+          <t>相关；相关性</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>El cuestionario mide actitudes lingüísticas.</t>
+          <t>Hay correlación entre horas de estudio y rendimiento.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>问卷测量语言态度。</t>
+          <t>学习时长与成绩之间存在相关。</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>images/cuestionario_1.jpg</t>
+          <t>images/correlacion_1.jpg</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2602,7 +2602,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>deducción</t>
+          <t>corroborar</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>v</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2622,34 +2622,34 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>演绎</t>
+          <t>证实；确证</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>La deducción parte de premisas generales.</t>
+          <t>Los datos corroboran la hipótesis.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>演绎从一般前提出发。</t>
+          <t>数据证实了该假设。</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>images/deduccion_1.jpg</t>
+          <t>images/corroborar_1.jpg</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>专八|专四</t>
+          <t>专八</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>delimitación</t>
+          <t>credibilidad</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2669,22 +2669,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>界定；划界</t>
+          <t>可信度</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>La delimitación del objeto de estudio es clave.</t>
+          <t>La fuente pierde credibilidad sin referencias.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>研究对象的界定很关键。</t>
+          <t>缺少出处会降低来源可信度。</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>images/delimitacion_1.jpg</t>
+          <t>images/credibilidad_1.jpg</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2696,7 +2696,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>demografía</t>
+          <t>criterio</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2716,34 +2716,34 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>人口学；人口结构</t>
+          <t>标准；准则；判断依据</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>La demografía explica cambios en el uso lingüístico.</t>
+          <t>El profesor utiliza varios criterios para evaluar la calidad de nuestros trabajos escritos.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>人口结构解释语言使用变化。</t>
+          <t>老师使用多种标准来评估我们书面作业的质量。</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>images/demografia_1.jpg</t>
+          <t>images/criterio_1.jpg</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>desplazamiento</t>
+          <t>crítica</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2763,22 +2763,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>迁移；转移</t>
+          <t>评论；批评</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>El desplazamiento semántico altera el significado.</t>
+          <t>La crítica literaria no solo juzga si un libro «gusta», sino cómo construye sentido y estilo.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>语义转移改变意义。</t>
+          <t>文学批评不只判断书是否「好看」，还分析它如何构建意义与风格。</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>images/desplazamiento_1.jpg</t>
+          <t>images/critica_1.jpg</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2790,7 +2790,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>dialecto</t>
+          <t>cuestionario</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2810,22 +2810,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>方言</t>
+          <t>问卷</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>El andaluz es un dialecto del español peninsular.</t>
+          <t>El cuestionario mide actitudes lingüísticas.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>安达卢西亚语是半岛西班牙语的一种方言。</t>
+          <t>问卷测量语言态度。</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>images/dialecto_1.jpg</t>
+          <t>images/cuestionario_1.jpg</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>dicotomía</t>
+          <t>deducción</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2857,34 +2857,34 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>二分法</t>
+          <t>推断；推论；演绎</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Evita una dicotomía demasiado rígida.</t>
+          <t>Tu deducción lógica sobre el final de la novela española sorprendió gratamente a toda la clase.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>避免过于僵硬的二分。</t>
+          <t>你对这部西班牙小说结局的逻辑推断让全班同学感到惊喜和钦佩。</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>images/dicotomia_1.jpg</t>
+          <t>images/deduccion_1.jpg</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>diferenciación</t>
+          <t>delimitación</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2904,22 +2904,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>分化；区分</t>
+          <t>界定；划界</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Hay diferenciación estilística entre géneros.</t>
+          <t>La delimitación del objeto de estudio es clave.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>体裁之间存在风格分化。</t>
+          <t>研究对象的界定很关键。</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>images/diferenciacion_1.jpg</t>
+          <t>images/delimitacion_1.jpg</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2931,7 +2931,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>discurso</t>
+          <t>demografía</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2951,22 +2951,22 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>话语；演说</t>
+          <t>人口学；人口结构</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>El discurso político usa metáforas y repeticiones para persuadir a una audiencia diversa.</t>
+          <t>La demografía explica cambios en el uso lingüístico.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>政治演说运用隐喻与重复，以说服多元听众。</t>
+          <t>人口结构解释语言使用变化。</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>images/discurso_1.jpg</t>
+          <t>images/demografia_1.jpg</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2978,7 +2978,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>distribución</t>
+          <t>desplazamiento</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2998,22 +2998,22 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>分布</t>
+          <t>迁移；转移</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Estudiamos la distribución geográfica del rasgo.</t>
+          <t>El desplazamiento semántico altera el significado.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>我们研究该特征的地理分布。</t>
+          <t>语义转移改变意义。</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>images/distribucion_1.jpg</t>
+          <t>images/desplazamiento_1.jpg</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3025,7 +3025,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>divergencia</t>
+          <t>dialecto</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3045,22 +3045,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>分歧；分化</t>
+          <t>方言</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>La divergencia dialectal aumenta con la distancia.</t>
+          <t>El andaluz es un dialecto del español peninsular.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>方言分歧随距离增大。</t>
+          <t>安达卢西亚语是半岛西班牙语的一种方言。</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>images/divergencia_1.jpg</t>
+          <t>images/dialecto_1.jpg</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3072,7 +3072,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>diversidad</t>
+          <t>dicotomía</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3092,22 +3092,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>多样性</t>
+          <t>二分法</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>La diversidad lingüística del mundo hispánico es un patrimonio que conviene preservar y estudiar.</t>
+          <t>Evita una dicotomía demasiado rígida.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>西语世界的语言多样性是值得保护与研究的遗产。</t>
+          <t>避免过于僵硬的二分。</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>images/diversidad_1.jpg</t>
+          <t>images/dicotomia_1.jpg</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3119,7 +3119,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>documentación</t>
+          <t>diferenciación</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3139,22 +3139,22 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>文献；文档工作</t>
+          <t>分化；区分</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>La documentación de lenguas en peligro es urgente.</t>
+          <t>Hay diferenciación estilística entre géneros.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>濒危语言文献工作紧迫。</t>
+          <t>体裁之间存在风格分化。</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>images/documentacion_1.jpg</t>
+          <t>images/diferenciacion_1.jpg</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3166,7 +3166,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>elaboración</t>
+          <t>discurso</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3186,22 +3186,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>加工；阐述</t>
+          <t>话语；演说</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>La elaboración del argumento requiere ejemplos.</t>
+          <t>El discurso político usa metáforas y repeticiones para persuadir a una audiencia diversa.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>论证的阐述需要例子。</t>
+          <t>政治演说运用隐喻与重复，以说服多元听众。</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>images/elaboracion_1.jpg</t>
+          <t>images/discurso_1.jpg</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3213,7 +3213,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>elipsis</t>
+          <t>distribución</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3233,22 +3233,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>省略</t>
+          <t>分布</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>La elipsis evita repeticiones innecesarias.</t>
+          <t>Estudiamos la distribución geográfica del rasgo.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>省略避免不必要的重复。</t>
+          <t>我们研究该特征的地理分布。</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>images/elipsis_1.jpg</t>
+          <t>images/distribucion_1.jpg</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3260,7 +3260,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>empatía</t>
+          <t>divergencia</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3280,22 +3280,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>共情</t>
+          <t>分歧；分化</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>La empatía del narrador acerca al lector.</t>
+          <t>La divergencia dialectal aumenta con la distancia.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>叙述者的共情拉近读者。</t>
+          <t>方言分歧随距离增大。</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>images/empatia_1.jpg</t>
+          <t>images/divergencia_1.jpg</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3307,7 +3307,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>encuesta</t>
+          <t>diversidad</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3327,22 +3327,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>调查</t>
+          <t>多样性</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>La encuesta recoge datos de percepción.</t>
+          <t>La diversidad lingüística del mundo hispánico es un patrimonio que conviene preservar y estudiar.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>调查收集感知数据。</t>
+          <t>西语世界的语言多样性是值得保护与研究的遗产。</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>images/encuesta_1.jpg</t>
+          <t>images/diversidad_1.jpg</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3354,7 +3354,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>enfoque</t>
+          <t>documentación</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3374,22 +3374,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>切入角度；方法焦点</t>
+          <t>文献；文档工作</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>El enfoque comunicativo prioriza el uso real de la lengua frente a la memorización de reglas.</t>
+          <t>La documentación de lenguas en peligro es urgente.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>交际法优先真实使用语言，而非死记规则。</t>
+          <t>濒危语言文献工作紧迫。</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>images/enfoque_1.jpg</t>
+          <t>images/documentacion_1.jpg</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3401,7 +3401,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>entorno</t>
+          <t>elaboración</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3421,22 +3421,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>环境；语境环境</t>
+          <t>加工；阐述</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>El entorno sociolingüístico condiciona el habla.</t>
+          <t>La elaboración del argumento requiere ejemplos.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>社会语言环境制约说话方式。</t>
+          <t>论证的阐述需要例子。</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>images/entorno_1.jpg</t>
+          <t>images/elaboracion_1.jpg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3448,7 +3448,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>enumeración</t>
+          <t>elipsis</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3468,22 +3468,22 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>列举</t>
+          <t>省略</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>La enumeración refuerza la idea principal.</t>
+          <t>La elipsis evita repeticiones innecesarias.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>列举强化中心思想。</t>
+          <t>省略避免不必要的重复。</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>images/enumeracion_1.jpg</t>
+          <t>images/elipsis_1.jpg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3495,7 +3495,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>enunciado</t>
+          <t>empatía</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3515,22 +3515,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>表述；话语单位</t>
+          <t>共情</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Cada enunciado realiza un acto de habla en contexto.</t>
+          <t>La empatía del narrador acerca al lector.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>每个表述在语境中完成一个言语行为。</t>
+          <t>叙述者的共情拉近读者。</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>images/enunciado_1.jpg</t>
+          <t>images/empatia_1.jpg</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3542,7 +3542,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>equivalencia</t>
+          <t>encuesta</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3562,22 +3562,22 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>对等</t>
+          <t>调查</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Busca equivalencia funcional en la traducción.</t>
+          <t>La encuesta recoge datos de percepción.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>翻译中寻求功能对等。</t>
+          <t>调查收集感知数据。</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>images/equivalencia_1.jpg</t>
+          <t>images/encuesta_1.jpg</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3589,7 +3589,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>escala</t>
+          <t>enfoque</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3609,22 +3609,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>量表；尺度</t>
+          <t>切入角度；方法焦点</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Usamos una escala Likert de cinco puntos.</t>
+          <t>El enfoque comunicativo prioriza el uso real de la lengua frente a la memorización de reglas.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>我们使用五点李克特量表。</t>
+          <t>交际法优先真实使用语言，而非死记规则。</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>images/escala_1.jpg</t>
+          <t>images/enfoque_1.jpg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3636,7 +3636,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>estabilidad</t>
+          <t>entorno</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3656,22 +3656,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>稳定性</t>
+          <t>环境；语境环境</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>La norma busca estabilidad ortográfica.</t>
+          <t>El entorno sociolingüístico condiciona el habla.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>规范追求拼写稳定。</t>
+          <t>社会语言环境制约说话方式。</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>images/estabilidad_1.jpg</t>
+          <t>images/entorno_1.jpg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3683,7 +3683,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>estigma</t>
+          <t>enumeración</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3703,22 +3703,22 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>污名</t>
+          <t>列举</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>El estigma lingüístico afecta a hablantes.</t>
+          <t>La enumeración refuerza la idea principal.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>语言污名影响使用者。</t>
+          <t>列举强化中心思想。</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>images/estigma_1.jpg</t>
+          <t>images/enumeracion_1.jpg</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3730,7 +3730,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>estilo</t>
+          <t>enunciado</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3750,22 +3750,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>风格；文风</t>
+          <t>表述；话语单位</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>El estilo del autor se reconoce por frases largas, adjetivos precisos y un humor contenido.</t>
+          <t>Cada enunciado realiza un acto de habla en contexto.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>作者的文风以长句、精确形容词与克制的幽默为特征。</t>
+          <t>每个表述在语境中完成一个言语行为。</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>images/estilo_1.jpg</t>
+          <t>images/enunciado_1.jpg</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3777,7 +3777,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>etnografía</t>
+          <t>equivalencia</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3797,22 +3797,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>民族志</t>
+          <t>对等</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>La etnografía observa prácticas situadas.</t>
+          <t>Busca equivalencia funcional en la traducción.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>民族志观察情境中的实践。</t>
+          <t>翻译中寻求功能对等。</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>images/etnografia_1.jpg</t>
+          <t>images/equivalencia_1.jpg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3824,7 +3824,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>evaluación</t>
+          <t>estigma</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3844,34 +3844,34 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>评价；评估</t>
+          <t>污名</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>La evaluación formativa guía el aprendizaje.</t>
+          <t>El estigma lingüístico afecta a hablantes.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>形成性评价引导学习。</t>
+          <t>语言污名影响使用者。</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>images/evaluacion_1.jpg</t>
+          <t>images/estigma_1.jpg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>专八|专四</t>
+          <t>专八</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>evidencia</t>
+          <t>estilo</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3891,22 +3891,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>证据</t>
+          <t>风格；文风</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>La evidencia empírica respalda la hipótesis principal.</t>
+          <t>El estilo del autor se reconoce por frases largas, adjetivos precisos y un humor contenido.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>经验证据支持主要假设。</t>
+          <t>作者的文风以长句、精确形容词与克制的幽默为特征。</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>images/evidencia_1.jpg</t>
+          <t>images/estilo_1.jpg</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3918,7 +3918,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>expectativa</t>
+          <t>etnografía</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3938,22 +3938,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>期待</t>
+          <t>民族志</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Rompe la expectativa del lector.</t>
+          <t>La etnografía observa prácticas situadas.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>它打破了读者的期待。</t>
+          <t>民族志观察情境中的实践。</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>images/expectativa_1.jpg</t>
+          <t>images/etnografia_1.jpg</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3965,7 +3965,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>explicación</t>
+          <t>evaluación</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3985,34 +3985,34 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>解释</t>
+          <t>评估；考试；评价</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>La explicación aclara el procedimiento.</t>
+          <t>La evaluación final del curso de español se basa tanto en la participación diaria como en el examen escrito.</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>解释澄清了步骤。</t>
+          <t>西语课程的期末评估既基于日常参与度，也基于笔试成绩。</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>images/explicacion_1.jpg</t>
+          <t>images/evaluacion_1.jpg</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>专八</t>
+          <t>专八|专四</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>exposición</t>
+          <t>expectativa</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4032,34 +4032,34 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>说明文；陈述</t>
+          <t>期待</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>La exposición presenta hechos con claridad.</t>
+          <t>Rompe la expectativa del lector.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>说明文清晰陈述事实。</t>
+          <t>它打破了读者的期待。</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>images/exposicion_1.jpg</t>
+          <t>images/expectativa_1.jpg</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>专八|专四</t>
+          <t>专八</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>fiabilidad</t>
+          <t>explicación</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4079,22 +4079,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>信度</t>
+          <t>解释</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Comprobamos la fiabilidad del instrumento.</t>
+          <t>La explicación aclara el procedimiento.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>我们检验工具信度。</t>
+          <t>解释澄清了步骤。</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>images/fiabilidad_1.jpg</t>
+          <t>images/explicacion_1.jpg</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>fonética</t>
+          <t>fiabilidad</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4126,22 +4126,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>语音学</t>
+          <t>信度</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>La fonética describe cómo se producen los sonidos.</t>
+          <t>Comprobamos la fiabilidad del instrumento.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>语音学描述语音如何发出。</t>
+          <t>我们检验工具信度。</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>images/fonetica_1.jpg</t>
+          <t>images/fiabilidad_1.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4153,7 +4153,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>fragmentación</t>
+          <t>fonética</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4173,22 +4173,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>碎片化</t>
+          <t>语音学</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>La fragmentación narrativa refleja crisis.</t>
+          <t>La fonética describe cómo se producen los sonidos.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>叙事碎片化反映危机。</t>
+          <t>语音学描述语音如何发出。</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>images/fragmentacion_1.jpg</t>
+          <t>images/fonetica_1.jpg</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4200,7 +4200,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>fuente</t>
+          <t>fragmentación</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4220,22 +4220,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>来源；（也指）泉水</t>
+          <t>碎片化</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Cita siempre la fuente primaria cuando uses datos estadísticos en tu trabajo de investigación.</t>
+          <t>La fragmentación narrativa refleja crisis.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>在研究作业中使用统计数据时，务必引用原始来源。</t>
+          <t>叙事碎片化反映危机。</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>images/fuente_1.jpg</t>
+          <t>images/fragmentacion_1.jpg</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4267,22 +4267,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>泉水；喷泉</t>
+          <t>来源；（也指）泉水</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Nos sentamos junto a la fuente de la plaza mientras repasábamos las preguntas del examen oral.</t>
+          <t>Cita siempre la fuente primaria cuando uses datos estadísticos en tu trabajo de investigación.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>我们坐在广场喷泉旁复习口语考试的问题。</t>
+          <t>在研究作业中使用统计数据时，务必引用原始来源。</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>images/fuente_2.jpg</t>
+          <t>images/fuente_1.jpg</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4294,12 +4294,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>generalización</t>
+          <t>fuente</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4314,22 +4314,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>概括</t>
+          <t>泉水；喷泉</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Evita generalizaciones apresuradas.</t>
+          <t>Nos sentamos junto a la fuente de la plaza mientras repasábamos las preguntas del examen oral.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>避免仓促概括。</t>
+          <t>我们坐在广场喷泉旁复习口语考试的问题。</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>images/generalizacion_1.jpg</t>
+          <t>images/fuente_2.jpg</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4341,7 +4341,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>globalización</t>
+          <t>generalización</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4361,22 +4361,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>全球化</t>
+          <t>概括</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>La globalización facilita el intercambio cultural, aunque también plantea retos a las identidades locales.</t>
+          <t>Evita generalizaciones apresuradas.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>全球化促进文化交流，同时也给地方认同带来挑战。</t>
+          <t>避免仓促概括。</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>images/globalizacion_1.jpg</t>
+          <t>images/generalizacion_1.jpg</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4388,7 +4388,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>glosario</t>
+          <t>globalización</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4408,22 +4408,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>术语表</t>
+          <t>全球化</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>El glosario define los términos técnicos del capítulo.</t>
+          <t>La globalización facilita el intercambio cultural, aunque también plantea retos a las identidades locales.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>术语表界定本章技术用语。</t>
+          <t>全球化促进文化交流，同时也给地方认同带来挑战。</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>images/glosario_1.jpg</t>
+          <t>images/globalizacion_1.jpg</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4435,7 +4435,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>hipotético</t>
+          <t>glosario</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>adj</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4455,22 +4455,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>假设的；假想的</t>
+          <t>术语表</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Partimos de un escenario hipotético para el debate.</t>
+          <t>El glosario define los términos técnicos del capítulo.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>我们从假想情景展开辩论。</t>
+          <t>术语表界定本章技术用语。</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>images/hipotetico_1.jpg</t>
+          <t>images/glosario_1.jpg</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4482,7 +4482,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>hipótesis</t>
+          <t>hipotético</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>adj</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4502,22 +4502,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>假设；假说</t>
+          <t>假设的；假想的</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>La hipótesis del estudio sostiene que el contacto frecuente con hablantes nativos acelera la fluidez.</t>
+          <t>Partimos de un escenario hipotético para el debate.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>该研究假设：与母语者频繁接触会加快流利度提升。</t>
+          <t>我们从假想情景展开辩论。</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>images/hipotesis_1.jpg</t>
+          <t>images/hipotetico_1.jpg</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -4529,7 +4529,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>homónimo</t>
+          <t>hipótesis</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4549,22 +4549,22 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>同音/同形异义词</t>
+          <t>假设；假说</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>«Banco» (asiento) y «banco» (entidad financiera) son homónimos: misma forma, sentidos distintos.</t>
+          <t>La hipótesis del estudio sostiene que el contacto frecuente con hablantes nativos acelera la fluidez.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>banco（长凳）与 banco（金融机构）是同形异义词：形式相同、意义不同。</t>
+          <t>该研究假设：与母语者频繁接触会加快流利度提升。</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>images/homonimo_1.jpg</t>
+          <t>images/hipotesis_1.jpg</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4576,7 +4576,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>identidad</t>
+          <t>homónimo</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4596,22 +4596,22 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>身份；认同</t>
+          <t>同音/同形异义词</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>La identidad cultural se construye con la lengua, la memoria familiar y las prácticas cotidianas.</t>
+          <t>«Banco» (asiento) y «banco» (entidad financiera) son homónimos: misma forma, sentidos distintos.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>文化认同由语言、家庭记忆与日常实践共同建构。</t>
+          <t>banco（长凳）与 banco（金融机构）是同形异义词：形式相同、意义不同。</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>images/identidad_1.jpg</t>
+          <t>images/homonimo_1.jpg</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -4623,7 +4623,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>inferencia</t>
+          <t>identidad</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4643,22 +4643,22 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>推断；推理</t>
+          <t>身份；认同</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Aunque el texto no lo diga explícitamente, por inferencia entendemos que el personaje está en crisis.</t>
+          <t>La identidad cultural se construye con la lengua, la memoria familiar y las prácticas cotidianas.</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>虽然文本未明说，通过推断我们明白人物正陷入危机。</t>
+          <t>文化认同由语言、家庭记忆与日常实践共同建构。</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>images/inferencia_1.jpg</t>
+          <t>images/identidad_1.jpg</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4670,7 +4670,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>innovación</t>
+          <t>inferencia</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4690,22 +4690,22 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>创新</t>
+          <t>推断；推理</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>La innovación educativa no es solo usar apps, sino rediseñar actividades para un aprendizaje activo.</t>
+          <t>Aunque el texto no lo diga explícitamente, por inferencia entendemos que el personaje está en crisis.</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>教育创新不只是用 App，而是重新设计活动以促进主动学习。</t>
+          <t>虽然文本未明说，通过推断我们明白人物正陷入危机。</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>images/innovacion_1.jpg</t>
+          <t>images/inferencia_1.jpg</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4717,7 +4717,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>interpretación</t>
+          <t>innovación</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4737,27 +4737,27 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>口译；解读</t>
+          <t>创新</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Su interpretación del poema destaca el tono irónico.</t>
+          <t>La innovación educativa no es solo usar apps, sino rediseñar actividades para un aprendizaje activo.</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>他对这首诗的解读突出了反讽语气。</t>
+          <t>教育创新不只是用 App，而是重新设计活动以促进主动学习。</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>images/interpretacion_1.jpg</t>
+          <t>images/innovacion_1.jpg</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>专八|专四</t>
+          <t>专八</t>
         </is>
       </c>
     </row>
@@ -5865,17 +5865,17 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>综合；综述</t>
+          <t>综合；总结；概要</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>La síntesis reúne las ideas principales sin detalles superfluos.</t>
+          <t>Hacer una síntesis de la lectura es una excelente estrategia para repasar la materia del examen.</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>综述汇总主要观点，不含多余细节。</t>
+          <t>对阅读内容做一份概要总结是复习考试科目的绝佳策略。</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">

</xml_diff>